<commit_message>
change drop box to select box
</commit_message>
<xml_diff>
--- a/backyard_list.xlsx
+++ b/backyard_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyApp\orderapp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A49ECA-8EAD-4A04-98BA-2C69F66BF6E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EFA228E-1510-46BA-8717-C423BA25D379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4A8513A4-3F40-4E3B-8380-35919E37163E}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="384">
-  <si>
-    <t>AE Spritz 1Dz</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="385">
   <si>
     <t>Sprtz Extrm 4oz</t>
   </si>
@@ -47,18 +44,12 @@
     <t>Sprtz Firm 4oz</t>
   </si>
   <si>
-    <t>AE Shine 4oz 1Dz / AE Herbal Oil 4oz 1Dz</t>
-  </si>
-  <si>
     <t>OilFree Spry 4oz</t>
   </si>
   <si>
     <t>H-Oil Spray 4oz</t>
   </si>
   <si>
-    <t>AE Lotion/Shampoo Dz / AE Spray 12oz Dz</t>
-  </si>
-  <si>
     <t>WrapStLtion4oz</t>
   </si>
   <si>
@@ -83,18 +74,12 @@
     <t>Weave Spry 12oz</t>
   </si>
   <si>
-    <t>SP BRAID SHEEN Shine Spray 12oz/1Dz</t>
-  </si>
-  <si>
     <t>Braid Sheen Argan 12oz</t>
   </si>
   <si>
     <t>Braid Sheen Keratin 12oz</t>
   </si>
   <si>
-    <t>SP HAIR FOOD 4 oz DZ</t>
-  </si>
-  <si>
     <t>Argan - (A)</t>
   </si>
   <si>
@@ -146,9 +131,6 @@
     <t>SP BLISTER -- FD</t>
   </si>
   <si>
-    <t>SP REMOVER LOTION / SHAMPOO</t>
-  </si>
-  <si>
     <t>RmvrLotion 2oz</t>
   </si>
   <si>
@@ -203,9 +185,6 @@
     <t>6dz S/P Glue1oz*6dz</t>
   </si>
   <si>
-    <t>30 LACE BOND REMOVER SYSTEM</t>
-  </si>
-  <si>
     <t>Extrm Bond 0.5oz</t>
   </si>
   <si>
@@ -242,9 +221,6 @@
     <t>Eyelash Glue WT 2oz</t>
   </si>
   <si>
-    <t>30 Strip Eyelash Glue 0.25oz Tube (Bulk) (36pcs)</t>
-  </si>
-  <si>
     <t>30Sec Eyelash Clear(Bulk)0.25o</t>
   </si>
   <si>
@@ -368,9 +344,6 @@
     <t>Jet Black4oz #130</t>
   </si>
   <si>
-    <t>VIA NATURAL Oil-Free WIG SHINE</t>
-  </si>
-  <si>
     <t>Wig Shine 8oz</t>
   </si>
   <si>
@@ -383,9 +356,6 @@
     <t>Wig Shine Dsply</t>
   </si>
   <si>
-    <t>VIA Tube Oil 24pc (100% Natural) 1display/master case, (VNCP24)</t>
-  </si>
-  <si>
     <t>Pro Growth 1.5oz</t>
   </si>
   <si>
@@ -440,9 +410,6 @@
     <t>Turmeric 1.5oz</t>
   </si>
   <si>
-    <t>VIA Tube Oil 3.5oz, 6pcs/display, 2display/case</t>
-  </si>
-  <si>
     <t>Via Tube Oil Biotin (3.5oz)</t>
   </si>
   <si>
@@ -470,9 +437,6 @@
     <t>Via Tube Oil Coconut (3.5oz)</t>
   </si>
   <si>
-    <t>VIA BRAIDING SHINE JELO (6pcs)</t>
-  </si>
-  <si>
     <t>Braiding Jelo 8oz</t>
   </si>
   <si>
@@ -488,9 +452,6 @@
     <t>ELIXIR BIOTIN 2OZ</t>
   </si>
   <si>
-    <t>VIA Premium Elixir Oil 2oz (6pcs)</t>
-  </si>
-  <si>
     <t>ELIXIR TEA TREE 2OZ</t>
   </si>
   <si>
@@ -533,9 +494,6 @@
     <t>Braid Display 24pc</t>
   </si>
   <si>
-    <t>VIA NATURAL PREMIUM STYLING GELS (6pcs)</t>
-  </si>
-  <si>
     <t>Olive w Aloe 8oz</t>
   </si>
   <si>
@@ -551,9 +509,6 @@
     <t>30 Eyelash WH 0.25&amp;1oz glu</t>
   </si>
   <si>
-    <t>30 Sec Eyelash 0.25 &amp; 1oz Glue Combo pack (24pcs)</t>
-  </si>
-  <si>
     <t>Beard Guyz</t>
   </si>
   <si>
@@ -677,9 +632,6 @@
     <t>JML Loc Unloc 16oz (6)</t>
   </si>
   <si>
-    <t>JML Cactus (6pcs)</t>
-  </si>
-  <si>
     <t>Cactus Oil Serum 4 oz</t>
   </si>
   <si>
@@ -692,18 +644,12 @@
     <t>Cactus Gro 6 oz</t>
   </si>
   <si>
-    <t>JML JBCO Shampoo and Conditioner (6pcs)</t>
-  </si>
-  <si>
     <t>Sulfate Free Sham 8oz</t>
   </si>
   <si>
     <t>Paraben Free Cond 8oz</t>
   </si>
   <si>
-    <t>NEW JML Black Castor Oil 2oz (6pcs/case)</t>
-  </si>
-  <si>
     <t>BCO Original 2oz (6)</t>
   </si>
   <si>
@@ -776,9 +722,6 @@
     <t>JBCO Peppermint 4oz</t>
   </si>
   <si>
-    <t>JML Black Castor Oil 8oz (6pcx)</t>
-  </si>
-  <si>
     <t>JML BCO Coconut 8oz</t>
   </si>
   <si>
@@ -794,9 +737,6 @@
     <t>JML 5n1 Lock Down 16oz</t>
   </si>
   <si>
-    <t>JML Minis Travel Size (24pcs)</t>
-  </si>
-  <si>
     <t>JML Tingle Shampoo 2oz</t>
   </si>
   <si>
@@ -818,9 +758,6 @@
     <t>JML No More Itch Spray 2oz</t>
   </si>
   <si>
-    <t>Robert Diamond Protective Shield</t>
-  </si>
-  <si>
     <t>Diamond Bond BK 2oz</t>
   </si>
   <si>
@@ -833,9 +770,6 @@
     <t>Diamond Bond Clear 8oz</t>
   </si>
   <si>
-    <t>Smooth Moisture Silkening System(JML)</t>
-  </si>
-  <si>
     <t>Silkening Shampoo 8oz</t>
   </si>
   <si>
@@ -893,9 +827,6 @@
     <t>JML 20pc Display Set</t>
   </si>
   <si>
-    <t>JML Boho (1oz Sample) &amp; BYW Combo (6pcs)</t>
-  </si>
-  <si>
     <t>JML Boho 1oz &amp; BYW Refresh</t>
   </si>
   <si>
@@ -923,15 +854,9 @@
     <t>JML Boho Fresh 8oz</t>
   </si>
   <si>
-    <t>JML Island Oil Gels 20oz (6pcs)</t>
-  </si>
-  <si>
     <t>Island Styling Jel 20oz</t>
   </si>
   <si>
-    <t>Hot Water Braid Dipper Jar (12pcs)</t>
-  </si>
-  <si>
     <t>JML Water Dipper(Sm)</t>
   </si>
   <si>
@@ -1178,16 +1103,94 @@
     <t>SP HAIR BONDING GLUE</t>
   </si>
   <si>
-    <t>30 Eyelash Glue 1dz Display</t>
-  </si>
-  <si>
-    <t>JML Wax and Gel (6pcs)</t>
-  </si>
-  <si>
-    <t>JML Sprays, Lotions, Shampoo, Conditioner (6pcs)</t>
-  </si>
-  <si>
-    <t>JML Black Castor Oil 4oz (6pcs)</t>
+    <t>AE Spritz</t>
+  </si>
+  <si>
+    <t>AE Shine/Herbal Oil</t>
+  </si>
+  <si>
+    <t>AE Lotion/Shampoo/Spray</t>
+  </si>
+  <si>
+    <t>SP BRAID SHEEN Shine Spray</t>
+  </si>
+  <si>
+    <t>SP HAIR FOOD</t>
+  </si>
+  <si>
+    <t>30 LACE BOND REMOVER</t>
+  </si>
+  <si>
+    <t>30 Eyelash Glue</t>
+  </si>
+  <si>
+    <t>30 Eyelash Glue 0.25oz Tube</t>
+  </si>
+  <si>
+    <t>VIA Oil-Free WIG SHINE</t>
+  </si>
+  <si>
+    <t>VIA Tube Oil 24pc</t>
+  </si>
+  <si>
+    <t>VIA Tube Oil 3.5oz</t>
+  </si>
+  <si>
+    <t>VIA BRAIDING SHINE JELO</t>
+  </si>
+  <si>
+    <t>VIA Premium Elixir Oil</t>
+  </si>
+  <si>
+    <t>VIA PREMIUM STYLING GELS</t>
+  </si>
+  <si>
+    <t>JML Wax and Gel</t>
+  </si>
+  <si>
+    <t>JML Loc Unloc</t>
+  </si>
+  <si>
+    <t>JML Cactus</t>
+  </si>
+  <si>
+    <t>JML Sp/Lo/Sh/Con</t>
+  </si>
+  <si>
+    <t>SP REMOVER LO/SH</t>
+  </si>
+  <si>
+    <t>30 Sec Eyelash &amp; Glue Combo</t>
+  </si>
+  <si>
+    <t>JML JBCO Sh/Con</t>
+  </si>
+  <si>
+    <t>NEW JML BCO 2oz</t>
+  </si>
+  <si>
+    <t>JML BCO 4oz</t>
+  </si>
+  <si>
+    <t>JML BCO 8oz</t>
+  </si>
+  <si>
+    <t>JML Minis Travel Size</t>
+  </si>
+  <si>
+    <t>Robert Diamond</t>
+  </si>
+  <si>
+    <t>Smooth Moisture</t>
+  </si>
+  <si>
+    <t>JML Boho &amp; BYW Combo</t>
+  </si>
+  <si>
+    <t>JML Island Oil Gels 20oz</t>
+  </si>
+  <si>
+    <t>Hot Water Braid Dipper Jar</t>
   </si>
 </sst>
 </file>
@@ -1615,24 +1618,24 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>364</v>
+        <v>339</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>365</v>
+        <v>340</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>366</v>
+        <v>341</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>367</v>
+        <v>342</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>1</v>
       </c>
       <c r="C2" s="4">
         <v>3504</v>
@@ -1643,10 +1646,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>0</v>
+        <v>355</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="4">
         <v>3404</v>
@@ -1657,10 +1660,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>356</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" s="4">
         <v>3304</v>
@@ -1671,10 +1674,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>5</v>
       </c>
       <c r="C5" s="4">
         <v>3904</v>
@@ -1685,10 +1688,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>357</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C6" s="4">
         <v>1204</v>
@@ -1699,10 +1702,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>357</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C7" s="4">
         <v>8109</v>
@@ -1713,10 +1716,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>9</v>
       </c>
       <c r="C8" s="4">
         <v>2512</v>
@@ -1727,10 +1730,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>6</v>
+        <v>357</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C9" s="4">
         <v>1012</v>
@@ -1741,10 +1744,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>6</v>
+        <v>357</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C10" s="4">
         <v>1207</v>
@@ -1755,10 +1758,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>6</v>
+        <v>357</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C11" s="4">
         <v>1312</v>
@@ -1769,10 +1772,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>6</v>
+        <v>357</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C12" s="4">
         <v>1404</v>
@@ -1783,10 +1786,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>6</v>
+        <v>357</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C13" s="4">
         <v>1412</v>
@@ -1797,10 +1800,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>15</v>
+        <v>358</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C14" s="4">
         <v>6838</v>
@@ -1811,10 +1814,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>15</v>
+        <v>358</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C15" s="4">
         <v>6839</v>
@@ -1825,10 +1828,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>18</v>
+        <v>359</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C16" s="4">
         <v>8102</v>
@@ -1839,10 +1842,10 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>18</v>
+        <v>359</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C17" s="4">
         <v>8103</v>
@@ -1853,10 +1856,10 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>18</v>
+        <v>359</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C18" s="4">
         <v>8104</v>
@@ -1867,13 +1870,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>18</v>
+        <v>359</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>302</v>
+        <v>277</v>
       </c>
       <c r="D19" s="3">
         <v>19.670000000000002</v>
@@ -1881,10 +1884,10 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="C20" s="4">
         <v>8114</v>
@@ -1895,10 +1898,10 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>18</v>
+        <v>359</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C21" s="4">
         <v>8113</v>
@@ -1909,10 +1912,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>18</v>
+        <v>359</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C22" s="4">
         <v>8108</v>
@@ -1923,10 +1926,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>18</v>
+        <v>359</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C23" s="4">
         <v>8111</v>
@@ -1937,10 +1940,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C24" s="4">
         <v>2001</v>
@@ -1951,10 +1954,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C25" s="4">
         <v>2002</v>
@@ -1965,10 +1968,10 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C26" s="4">
         <v>2003</v>
@@ -1979,10 +1982,10 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C27" s="4">
         <v>2443</v>
@@ -1993,13 +1996,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D28" s="3">
         <v>21.6</v>
@@ -2007,10 +2010,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C29" s="4">
         <v>2103</v>
@@ -2021,10 +2024,10 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C30" s="4">
         <v>2441</v>
@@ -2035,10 +2038,10 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C31" s="4">
         <v>2005</v>
@@ -2049,10 +2052,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C32" s="4">
         <v>2102</v>
@@ -2063,10 +2066,10 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>36</v>
+        <v>373</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C33" s="4">
         <v>2202</v>
@@ -2077,10 +2080,10 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>36</v>
+        <v>373</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C34" s="4">
         <v>2204</v>
@@ -2091,10 +2094,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>36</v>
+        <v>373</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C35" s="4">
         <v>2305</v>
@@ -2105,10 +2108,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>36</v>
+        <v>373</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C36" s="4">
         <v>2306</v>
@@ -2119,10 +2122,10 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C37" s="4">
         <v>2416</v>
@@ -2133,10 +2136,10 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C38" s="4">
         <v>2415</v>
@@ -2147,10 +2150,10 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C39" s="4">
         <v>2409</v>
@@ -2161,10 +2164,10 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C40" s="4">
         <v>2448</v>
@@ -2175,10 +2178,10 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C41" s="4">
         <v>2410</v>
@@ -2189,10 +2192,10 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C42" s="4">
         <v>2411</v>
@@ -2203,10 +2206,10 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C43" s="4">
         <v>2413</v>
@@ -2217,10 +2220,10 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C44" s="4">
         <v>2404</v>
@@ -2231,10 +2234,10 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C45" s="4">
         <v>2408</v>
@@ -2245,10 +2248,10 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C46" s="4">
         <v>2414</v>
@@ -2259,10 +2262,10 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C47" s="4">
         <v>2446</v>
@@ -2273,10 +2276,10 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C48" s="4">
         <v>2440</v>
@@ -2287,10 +2290,10 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C49" s="4">
         <v>2407</v>
@@ -2301,10 +2304,10 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C50" s="4">
         <v>2421</v>
@@ -2315,10 +2318,10 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>55</v>
+        <v>360</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C51" s="4">
         <v>2540</v>
@@ -2329,10 +2332,10 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>55</v>
+        <v>360</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C52" s="4">
         <v>2621</v>
@@ -2343,10 +2346,10 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>55</v>
+        <v>360</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C53" s="4">
         <v>2620</v>
@@ -2357,10 +2360,10 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C54" s="4">
         <v>8636</v>
@@ -2371,10 +2374,10 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C55" s="4">
         <v>8638</v>
@@ -2385,10 +2388,10 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C56" s="4">
         <v>8635</v>
@@ -2399,10 +2402,10 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C57" s="4">
         <v>8637</v>
@@ -2413,10 +2416,10 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>380</v>
+        <v>361</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C58" s="4">
         <v>81862</v>
@@ -2427,10 +2430,10 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>380</v>
+        <v>361</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C59" s="4">
         <v>81864</v>
@@ -2441,10 +2444,10 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>380</v>
+        <v>361</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C60" s="4">
         <v>81861</v>
@@ -2455,10 +2458,10 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>380</v>
+        <v>361</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C61" s="4">
         <v>81863</v>
@@ -2469,10 +2472,10 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>68</v>
+        <v>362</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C62" s="4">
         <v>24683</v>
@@ -2483,10 +2486,10 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>68</v>
+        <v>362</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C63" s="4">
         <v>24693</v>
@@ -2497,10 +2500,10 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C64" s="4">
         <v>2555</v>
@@ -2511,10 +2514,10 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C65" s="4">
         <v>2557</v>
@@ -2525,10 +2528,10 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="C66" s="4">
         <v>2556</v>
@@ -2539,10 +2542,10 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="C67" s="4">
         <v>2558</v>
@@ -2553,13 +2556,13 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>303</v>
+        <v>278</v>
       </c>
       <c r="D68" s="3">
         <v>8.34</v>
@@ -2567,13 +2570,13 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>304</v>
+        <v>279</v>
       </c>
       <c r="D69" s="3">
         <v>8.34</v>
@@ -2581,13 +2584,13 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>305</v>
+        <v>280</v>
       </c>
       <c r="D70" s="3">
         <v>8.34</v>
@@ -2595,13 +2598,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>306</v>
+        <v>281</v>
       </c>
       <c r="D71" s="3">
         <v>8.34</v>
@@ -2609,13 +2612,13 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>307</v>
+        <v>282</v>
       </c>
       <c r="D72" s="3">
         <v>8.34</v>
@@ -2623,13 +2626,13 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>308</v>
+        <v>283</v>
       </c>
       <c r="D73" s="3">
         <v>8.34</v>
@@ -2637,13 +2640,13 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>309</v>
+        <v>284</v>
       </c>
       <c r="D74" s="3">
         <v>8.34</v>
@@ -2651,13 +2654,13 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B75" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B75" s="6" t="s">
-        <v>84</v>
-      </c>
       <c r="C75" s="4" t="s">
-        <v>310</v>
+        <v>285</v>
       </c>
       <c r="D75" s="3">
         <v>8.34</v>
@@ -2665,13 +2668,13 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>311</v>
+        <v>286</v>
       </c>
       <c r="D76" s="3">
         <v>8.34</v>
@@ -2679,13 +2682,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>312</v>
+        <v>287</v>
       </c>
       <c r="D77" s="3">
         <v>8.34</v>
@@ -2693,13 +2696,13 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>313</v>
+        <v>288</v>
       </c>
       <c r="D78" s="3">
         <v>8.34</v>
@@ -2707,13 +2710,13 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>314</v>
+        <v>289</v>
       </c>
       <c r="D79" s="3">
         <v>8.34</v>
@@ -2721,13 +2724,13 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>315</v>
+        <v>290</v>
       </c>
       <c r="D80" s="3">
         <v>8.34</v>
@@ -2735,13 +2738,13 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>316</v>
+        <v>291</v>
       </c>
       <c r="D81" s="3">
         <v>8.34</v>
@@ -2749,13 +2752,13 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>317</v>
+        <v>292</v>
       </c>
       <c r="D82" s="3">
         <v>8.34</v>
@@ -2763,13 +2766,13 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>318</v>
+        <v>293</v>
       </c>
       <c r="D83" s="3">
         <v>8.34</v>
@@ -2777,13 +2780,13 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>319</v>
+        <v>294</v>
       </c>
       <c r="D84" s="3">
         <v>14.46</v>
@@ -2791,13 +2794,13 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>320</v>
+        <v>295</v>
       </c>
       <c r="D85" s="3">
         <v>14.46</v>
@@ -2805,13 +2808,13 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="D86" s="3">
         <v>14.46</v>
@@ -2819,13 +2822,13 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>322</v>
+        <v>297</v>
       </c>
       <c r="D87" s="3">
         <v>14.46</v>
@@ -2833,13 +2836,13 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>323</v>
+        <v>298</v>
       </c>
       <c r="D88" s="3">
         <v>14.46</v>
@@ -2847,13 +2850,13 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>324</v>
+        <v>299</v>
       </c>
       <c r="D89" s="3">
         <v>14.46</v>
@@ -2861,13 +2864,13 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>325</v>
+        <v>300</v>
       </c>
       <c r="D90" s="3">
         <v>14.46</v>
@@ -2875,13 +2878,13 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>326</v>
+        <v>301</v>
       </c>
       <c r="D91" s="3">
         <v>14.46</v>
@@ -2889,13 +2892,13 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B92" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B92" s="5" t="s">
-        <v>102</v>
-      </c>
       <c r="C92" s="4" t="s">
-        <v>327</v>
+        <v>302</v>
       </c>
       <c r="D92" s="3">
         <v>14.46</v>
@@ -2903,13 +2906,13 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>328</v>
+        <v>303</v>
       </c>
       <c r="D93" s="3">
         <v>14.46</v>
@@ -2917,13 +2920,13 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="D94" s="3">
         <v>14.46</v>
@@ -2931,13 +2934,13 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>330</v>
+        <v>305</v>
       </c>
       <c r="D95" s="3">
         <v>14.46</v>
@@ -2945,13 +2948,13 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>331</v>
+        <v>306</v>
       </c>
       <c r="D96" s="3">
         <v>14.46</v>
@@ -2959,13 +2962,13 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>332</v>
+        <v>307</v>
       </c>
       <c r="D97" s="3">
         <v>14.46</v>
@@ -2973,13 +2976,13 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>333</v>
+        <v>308</v>
       </c>
       <c r="D98" s="3">
         <v>14.46</v>
@@ -2987,13 +2990,13 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>334</v>
+        <v>309</v>
       </c>
       <c r="D99" s="3">
         <v>14.46</v>
@@ -3001,10 +3004,10 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="C100" s="4">
         <v>8351</v>
@@ -3015,10 +3018,10 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="C101" s="4">
         <v>8352</v>
@@ -3029,10 +3032,10 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="C102" s="4">
         <v>8353</v>
@@ -3043,10 +3046,10 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>110</v>
+        <v>363</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="C103" s="4">
         <v>8354</v>
@@ -3057,10 +3060,10 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C104" s="4">
         <v>57974</v>
@@ -3071,10 +3074,10 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C105" s="4">
         <v>57975</v>
@@ -3085,10 +3088,10 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C106" s="4">
         <v>57976</v>
@@ -3099,10 +3102,10 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C107" s="4">
         <v>57977</v>
@@ -3113,10 +3116,10 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C108" s="4">
         <v>57978</v>
@@ -3127,10 +3130,10 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C109" s="4">
         <v>57979</v>
@@ -3141,10 +3144,10 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C110" s="4">
         <v>57980</v>
@@ -3155,10 +3158,10 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C111" s="4">
         <v>57981</v>
@@ -3169,10 +3172,10 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C112" s="4">
         <v>57982</v>
@@ -3183,10 +3186,10 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C113" s="4">
         <v>57983</v>
@@ -3197,10 +3200,10 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="B114" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="C114" s="4">
         <v>57984</v>
@@ -3211,10 +3214,10 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C115" s="4">
         <v>57985</v>
@@ -3225,10 +3228,10 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C116" s="4">
         <v>57986</v>
@@ -3239,10 +3242,10 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C117" s="4">
         <v>57987</v>
@@ -3253,10 +3256,10 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C118" s="4">
         <v>57988</v>
@@ -3267,10 +3270,10 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C119" s="4">
         <v>57989</v>
@@ -3281,10 +3284,10 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="C120" s="4">
         <v>57990</v>
@@ -3295,10 +3298,10 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="C121" s="4">
         <v>57991</v>
@@ -3309,10 +3312,10 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
-        <v>115</v>
+        <v>364</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C122" s="4">
         <v>58000</v>
@@ -3323,10 +3326,10 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="C123" s="4">
         <v>58001</v>
@@ -3337,10 +3340,10 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="C124" s="4">
         <v>58002</v>
@@ -3351,10 +3354,10 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="C125" s="4">
         <v>58003</v>
@@ -3365,10 +3368,10 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="C126" s="4">
         <v>58004</v>
@@ -3379,10 +3382,10 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="C127" s="4">
         <v>58005</v>
@@ -3393,10 +3396,10 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C128" s="4">
         <v>58006</v>
@@ -3407,10 +3410,10 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C129" s="4">
         <v>58007</v>
@@ -3421,10 +3424,10 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
-        <v>134</v>
+        <v>365</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="C130" s="4">
         <v>58008</v>
@@ -3435,10 +3438,10 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
-        <v>144</v>
+        <v>366</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C131" s="4">
         <v>8390</v>
@@ -3449,10 +3452,10 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
-        <v>144</v>
+        <v>366</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="C132" s="4">
         <v>8393</v>
@@ -3463,10 +3466,10 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
-        <v>144</v>
+        <v>366</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="C133" s="4">
         <v>8392</v>
@@ -3477,10 +3480,10 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
-        <v>144</v>
+        <v>366</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="C134" s="4">
         <v>8394</v>
@@ -3491,10 +3494,10 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="C135" s="4">
         <v>81872</v>
@@ -3505,10 +3508,10 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="C136" s="4">
         <v>81874</v>
@@ -3519,10 +3522,10 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="C137" s="4">
         <v>81876</v>
@@ -3533,10 +3536,10 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="C138" s="4">
         <v>81873</v>
@@ -3547,10 +3550,10 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="C139" s="4">
         <v>81875</v>
@@ -3561,10 +3564,10 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="C140" s="4">
         <v>81877</v>
@@ -3575,10 +3578,10 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
-        <v>150</v>
+        <v>367</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="C141" s="4">
         <v>81916</v>
@@ -3589,10 +3592,10 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="C142" s="4">
         <v>1899</v>
@@ -3603,10 +3606,10 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="C143" s="4">
         <v>1900</v>
@@ -3617,10 +3620,10 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="3" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="C144" s="4">
         <v>1901</v>
@@ -3631,10 +3634,10 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="C145" s="4">
         <v>1902</v>
@@ -3645,10 +3648,10 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="3" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="C146" s="4">
         <v>1903</v>
@@ -3659,10 +3662,10 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="C147" s="4">
         <v>1904</v>
@@ -3673,10 +3676,10 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="C148" s="4">
         <v>1905</v>
@@ -3687,10 +3690,10 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
-        <v>165</v>
+        <v>368</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="C149" s="4">
         <v>8380</v>
@@ -3701,10 +3704,10 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
-        <v>165</v>
+        <v>368</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="C150" s="4">
         <v>8385</v>
@@ -3715,10 +3718,10 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
-        <v>165</v>
+        <v>368</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="C151" s="4">
         <v>8384</v>
@@ -3729,10 +3732,10 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
-        <v>165</v>
+        <v>368</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="C152" s="4">
         <v>8389</v>
@@ -3743,10 +3746,10 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="5" t="s">
-        <v>171</v>
+        <v>374</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="C153" s="4">
         <v>24696</v>
@@ -3757,13 +3760,13 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>368</v>
+        <v>343</v>
       </c>
       <c r="D154" s="3">
         <v>37.76</v>
@@ -3771,13 +3774,13 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>369</v>
+        <v>344</v>
       </c>
       <c r="D155" s="3">
         <v>37.76</v>
@@ -3785,13 +3788,13 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B156" s="6" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>370</v>
+        <v>345</v>
       </c>
       <c r="D156" s="3">
         <v>194.24</v>
@@ -3799,13 +3802,13 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B157" s="6" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>371</v>
+        <v>346</v>
       </c>
       <c r="D157" s="3">
         <v>194.24</v>
@@ -3813,13 +3816,13 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>372</v>
+        <v>347</v>
       </c>
       <c r="D158" s="3">
         <v>75.52</v>
@@ -3827,13 +3830,13 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B159" s="6" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>373</v>
+        <v>348</v>
       </c>
       <c r="D159" s="3">
         <v>194.24</v>
@@ -3841,13 +3844,13 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>374</v>
+        <v>349</v>
       </c>
       <c r="D160" s="3">
         <v>75.52</v>
@@ -3855,13 +3858,13 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B161" s="6" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>375</v>
+        <v>350</v>
       </c>
       <c r="D161" s="3">
         <v>75.52</v>
@@ -3869,13 +3872,13 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>376</v>
+        <v>351</v>
       </c>
       <c r="D162" s="3">
         <v>75.52</v>
@@ -3883,13 +3886,13 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>377</v>
+        <v>352</v>
       </c>
       <c r="D163" s="3">
         <v>151.04</v>
@@ -3897,10 +3900,10 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="C164" s="4">
         <v>29080</v>
@@ -3911,10 +3914,10 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="C165" s="4">
         <v>29085</v>
@@ -3925,10 +3928,10 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="C166" s="4">
         <v>29401</v>
@@ -3939,10 +3942,10 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="C167" s="4">
         <v>29402</v>
@@ -3953,10 +3956,10 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="C168" s="4">
         <v>29420</v>
@@ -3967,10 +3970,10 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B169" s="5" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="C169" s="4">
         <v>29050</v>
@@ -3981,10 +3984,10 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B170" s="5" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="C170" s="4">
         <v>29055</v>
@@ -3995,10 +3998,10 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B171" s="5" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="C171" s="4">
         <v>29020</v>
@@ -4009,10 +4012,10 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B172" s="6" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="C172" s="4">
         <v>29010</v>
@@ -4023,10 +4026,10 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B173" s="5" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="C173" s="4">
         <v>29093</v>
@@ -4037,10 +4040,10 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B174" s="5" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="C174" s="4">
         <v>29302</v>
@@ -4051,10 +4054,10 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B175" s="5" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="C175" s="4">
         <v>29407</v>
@@ -4065,10 +4068,10 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B176" s="5" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="C176" s="4">
         <v>29405</v>
@@ -4079,10 +4082,10 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="3" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B177" s="5" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="C177" s="4">
         <v>29409</v>
@@ -4093,10 +4096,10 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B178" s="5" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="C178" s="4">
         <v>29030</v>
@@ -4107,10 +4110,10 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B179" s="5" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="C179" s="4">
         <v>29406</v>
@@ -4121,10 +4124,10 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B180" s="5" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="C180" s="4">
         <v>29304</v>
@@ -4135,10 +4138,10 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B181" s="5" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="C181" s="4">
         <v>29300</v>
@@ -4149,10 +4152,10 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C182" s="4">
         <v>29060</v>
@@ -4163,10 +4166,10 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B183" s="5" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C183" s="4">
         <v>29066</v>
@@ -4177,10 +4180,10 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B184" s="5" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C184" s="4">
         <v>29070</v>
@@ -4191,10 +4194,10 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B185" s="5" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C185" s="4">
         <v>29076</v>
@@ -4205,10 +4208,10 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B186" s="5" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C186" s="4">
         <v>29040</v>
@@ -4219,10 +4222,10 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B187" s="5" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C187" s="4">
         <v>29042</v>
@@ -4233,10 +4236,10 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B188" s="5" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C188" s="4">
         <v>29041</v>
@@ -4247,10 +4250,10 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B189" s="5" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="C189" s="4">
         <v>29043</v>
@@ -4261,10 +4264,10 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B190" s="6" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="C190" s="4">
         <v>29092</v>
@@ -4275,10 +4278,10 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B191" s="5" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="C191" s="4">
         <v>29094</v>
@@ -4289,10 +4292,10 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="3" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B192" s="5" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="C192" s="4">
         <v>29404</v>
@@ -4303,10 +4306,10 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" s="3" t="s">
-        <v>212</v>
+        <v>370</v>
       </c>
       <c r="B193" s="5" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="C193" s="4">
         <v>81921</v>
@@ -4317,10 +4320,10 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="3" t="s">
-        <v>213</v>
+        <v>371</v>
       </c>
       <c r="B194" s="5" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="C194" s="4">
         <v>29098</v>
@@ -4331,10 +4334,10 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" s="3" t="s">
-        <v>213</v>
+        <v>371</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="C195" s="4">
         <v>29095</v>
@@ -4345,10 +4348,10 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" s="3" t="s">
-        <v>213</v>
+        <v>371</v>
       </c>
       <c r="B196" s="5" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C196" s="4">
         <v>29096</v>
@@ -4359,10 +4362,10 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" s="3" t="s">
-        <v>213</v>
+        <v>371</v>
       </c>
       <c r="B197" s="5" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C197" s="4">
         <v>29097</v>
@@ -4373,13 +4376,13 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" s="3" t="s">
-        <v>218</v>
+        <v>375</v>
       </c>
       <c r="B198" s="5" t="s">
-        <v>219</v>
+        <v>202</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>335</v>
+        <v>310</v>
       </c>
       <c r="D198" s="3">
         <v>0</v>
@@ -4387,13 +4390,13 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" s="3" t="s">
-        <v>218</v>
+        <v>375</v>
       </c>
       <c r="B199" s="5" t="s">
-        <v>220</v>
+        <v>203</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>336</v>
+        <v>311</v>
       </c>
       <c r="D199" s="3">
         <v>0</v>
@@ -4401,13 +4404,13 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B200" s="5" t="s">
-        <v>222</v>
+        <v>204</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>337</v>
+        <v>312</v>
       </c>
       <c r="D200" s="3">
         <v>20.16</v>
@@ -4415,13 +4418,13 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B201" s="5" t="s">
-        <v>223</v>
+        <v>205</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>338</v>
+        <v>313</v>
       </c>
       <c r="D201" s="3">
         <v>20.16</v>
@@ -4429,13 +4432,13 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B202" s="5" t="s">
-        <v>224</v>
+        <v>206</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>339</v>
+        <v>314</v>
       </c>
       <c r="D202" s="3">
         <v>20.16</v>
@@ -4443,13 +4446,13 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B203" s="5" t="s">
-        <v>225</v>
+        <v>207</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
       <c r="D203" s="3">
         <v>20.16</v>
@@ -4457,13 +4460,13 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B204" s="5" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="C204" s="4" t="s">
-        <v>341</v>
+        <v>316</v>
       </c>
       <c r="D204" s="3">
         <v>20.16</v>
@@ -4471,13 +4474,13 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B205" s="5" t="s">
-        <v>227</v>
+        <v>209</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>342</v>
+        <v>317</v>
       </c>
       <c r="D205" s="3">
         <v>20.16</v>
@@ -4485,13 +4488,13 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B206" s="5" t="s">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>343</v>
+        <v>318</v>
       </c>
       <c r="D206" s="3">
         <v>20.16</v>
@@ -4499,13 +4502,13 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>344</v>
+        <v>319</v>
       </c>
       <c r="D207" s="3">
         <v>20.16</v>
@@ -4513,13 +4516,13 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B208" s="5" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="C208" s="4" t="s">
-        <v>345</v>
+        <v>320</v>
       </c>
       <c r="D208" s="3">
         <v>20.16</v>
@@ -4527,13 +4530,13 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B209" s="5" t="s">
-        <v>231</v>
+        <v>213</v>
       </c>
       <c r="C209" s="4" t="s">
-        <v>346</v>
+        <v>321</v>
       </c>
       <c r="D209" s="3">
         <v>20.16</v>
@@ -4541,13 +4544,13 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B210" s="5" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="C210" s="4" t="s">
-        <v>347</v>
+        <v>322</v>
       </c>
       <c r="D210" s="3">
         <v>20.16</v>
@@ -4555,13 +4558,13 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" s="3" t="s">
-        <v>221</v>
+        <v>376</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>233</v>
+        <v>215</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>348</v>
+        <v>323</v>
       </c>
       <c r="D211" s="3">
         <v>20.16</v>
@@ -4569,13 +4572,13 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B212" s="5" t="s">
-        <v>234</v>
+        <v>216</v>
       </c>
       <c r="C212" s="4" t="s">
-        <v>349</v>
+        <v>324</v>
       </c>
       <c r="D212" s="3">
         <v>34.24</v>
@@ -4583,13 +4586,13 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B213" s="5" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="C213" s="4" t="s">
-        <v>350</v>
+        <v>325</v>
       </c>
       <c r="D213" s="3">
         <v>34.24</v>
@@ -4597,13 +4600,13 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B214" s="5" t="s">
-        <v>236</v>
+        <v>218</v>
       </c>
       <c r="C214" s="4" t="s">
-        <v>351</v>
+        <v>326</v>
       </c>
       <c r="D214" s="3">
         <v>34.24</v>
@@ -4611,13 +4614,13 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
       <c r="C215" s="4" t="s">
-        <v>352</v>
+        <v>327</v>
       </c>
       <c r="D215" s="3">
         <v>34.24</v>
@@ -4625,13 +4628,13 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="C216" s="4" t="s">
-        <v>353</v>
+        <v>328</v>
       </c>
       <c r="D216" s="3">
         <v>34.24</v>
@@ -4639,13 +4642,13 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="C217" s="4" t="s">
-        <v>354</v>
+        <v>329</v>
       </c>
       <c r="D217" s="3">
         <v>34.24</v>
@@ -4653,13 +4656,13 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>355</v>
+        <v>330</v>
       </c>
       <c r="D218" s="3">
         <v>34.24</v>
@@ -4667,13 +4670,13 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>356</v>
+        <v>331</v>
       </c>
       <c r="D219" s="3">
         <v>34.24</v>
@@ -4681,13 +4684,13 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B220" s="5" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>357</v>
+        <v>332</v>
       </c>
       <c r="D220" s="3">
         <v>34.24</v>
@@ -4695,13 +4698,13 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B221" s="5" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>358</v>
+        <v>333</v>
       </c>
       <c r="D221" s="3">
         <v>34.24</v>
@@ -4709,13 +4712,13 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>359</v>
+        <v>334</v>
       </c>
       <c r="D222" s="3">
         <v>34.24</v>
@@ -4723,13 +4726,13 @@
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>245</v>
+        <v>227</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>360</v>
+        <v>335</v>
       </c>
       <c r="D223" s="3">
         <v>34.24</v>
@@ -4737,13 +4740,13 @@
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" s="3" t="s">
-        <v>246</v>
+        <v>378</v>
       </c>
       <c r="B224" s="5" t="s">
-        <v>247</v>
+        <v>228</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>361</v>
+        <v>336</v>
       </c>
       <c r="D224" s="3">
         <v>0</v>
@@ -4751,13 +4754,13 @@
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" s="3" t="s">
-        <v>246</v>
+        <v>378</v>
       </c>
       <c r="B225" s="5" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>362</v>
+        <v>337</v>
       </c>
       <c r="D225" s="3">
         <v>0</v>
@@ -4765,13 +4768,13 @@
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" s="3" t="s">
-        <v>246</v>
+        <v>378</v>
       </c>
       <c r="B226" s="5" t="s">
-        <v>249</v>
+        <v>230</v>
       </c>
       <c r="C226" s="4" t="s">
-        <v>363</v>
+        <v>338</v>
       </c>
       <c r="D226" s="3">
         <v>0</v>
@@ -4779,10 +4782,10 @@
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" s="3" t="s">
-        <v>250</v>
+        <v>231</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>251</v>
+        <v>232</v>
       </c>
       <c r="C227" s="4">
         <v>81034</v>
@@ -4793,10 +4796,10 @@
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" s="3" t="s">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="C228" s="4">
         <v>81925</v>
@@ -4807,10 +4810,10 @@
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" s="3" t="s">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="C229" s="4">
         <v>81927</v>
@@ -4821,10 +4824,10 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" s="3" t="s">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="B230" s="5" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="C230" s="4">
         <v>81929</v>
@@ -4835,10 +4838,10 @@
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" s="3" t="s">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="B231" s="5" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="C231" s="4">
         <v>81033</v>
@@ -4849,10 +4852,10 @@
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" s="3" t="s">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="B232" s="5" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
       <c r="C232" s="4">
         <v>81926</v>
@@ -4863,10 +4866,10 @@
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" s="3" t="s">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="C233" s="4">
         <v>81928</v>
@@ -4877,10 +4880,10 @@
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" s="3" t="s">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="B234" s="5" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="C234" s="4">
         <v>81932</v>
@@ -4891,10 +4894,10 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" s="3" t="s">
-        <v>260</v>
+        <v>380</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>261</v>
+        <v>240</v>
       </c>
       <c r="C235" s="4">
         <v>3060</v>
@@ -4905,10 +4908,10 @@
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" s="3" t="s">
-        <v>260</v>
+        <v>380</v>
       </c>
       <c r="B236" s="5" t="s">
-        <v>262</v>
+        <v>241</v>
       </c>
       <c r="C236" s="4">
         <v>3062</v>
@@ -4919,10 +4922,10 @@
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" s="3" t="s">
-        <v>260</v>
+        <v>380</v>
       </c>
       <c r="B237" s="5" t="s">
-        <v>263</v>
+        <v>242</v>
       </c>
       <c r="C237" s="4">
         <v>3059</v>
@@ -4933,10 +4936,10 @@
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" s="3" t="s">
-        <v>260</v>
+        <v>380</v>
       </c>
       <c r="B238" s="5" t="s">
-        <v>264</v>
+        <v>243</v>
       </c>
       <c r="C238" s="4">
         <v>3061</v>
@@ -4947,10 +4950,10 @@
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" s="3" t="s">
-        <v>265</v>
+        <v>381</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="C239" s="4">
         <v>1850</v>
@@ -4961,10 +4964,10 @@
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" s="3" t="s">
-        <v>265</v>
+        <v>381</v>
       </c>
       <c r="B240" s="5" t="s">
-        <v>267</v>
+        <v>245</v>
       </c>
       <c r="C240" s="4">
         <v>1851</v>
@@ -4975,10 +4978,10 @@
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" s="3" t="s">
-        <v>265</v>
+        <v>381</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="C241" s="4">
         <v>1852</v>
@@ -4989,10 +4992,10 @@
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" s="3" t="s">
-        <v>265</v>
+        <v>381</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>269</v>
+        <v>247</v>
       </c>
       <c r="C242" s="4">
         <v>1853</v>
@@ -5003,10 +5006,10 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" s="3" t="s">
-        <v>265</v>
+        <v>381</v>
       </c>
       <c r="B243" s="5" t="s">
-        <v>270</v>
+        <v>248</v>
       </c>
       <c r="C243" s="4">
         <v>1856</v>
@@ -5017,10 +5020,10 @@
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" s="3" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B244" s="5" t="s">
-        <v>272</v>
+        <v>250</v>
       </c>
       <c r="C244" s="4">
         <v>76081</v>
@@ -5031,10 +5034,10 @@
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" s="3" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B245" s="5" t="s">
-        <v>273</v>
+        <v>251</v>
       </c>
       <c r="C245" s="4">
         <v>76085</v>
@@ -5045,10 +5048,10 @@
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" s="3" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B246" s="5" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
       <c r="C246" s="4">
         <v>76087</v>
@@ -5059,10 +5062,10 @@
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" s="3" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="C247" s="4">
         <v>76082</v>
@@ -5073,10 +5076,10 @@
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" s="3" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="C248" s="4">
         <v>76086</v>
@@ -5087,10 +5090,10 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="C249" s="4">
         <v>1015</v>
@@ -5101,10 +5104,10 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
       <c r="C250" s="4">
         <v>1016</v>
@@ -5115,10 +5118,10 @@
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="C251" s="4">
         <v>1017</v>
@@ -5129,10 +5132,10 @@
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="B252" s="5" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="C252" s="4">
         <v>1022</v>
@@ -5143,10 +5146,10 @@
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="C253" s="4">
         <v>1018</v>
@@ -5157,10 +5160,10 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="B254" s="5" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="C254" s="4">
         <v>1019</v>
@@ -5171,10 +5174,10 @@
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" s="3" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="C255" s="4">
         <v>1020</v>
@@ -5185,10 +5188,10 @@
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" s="3" t="s">
-        <v>285</v>
+        <v>382</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>286</v>
+        <v>263</v>
       </c>
       <c r="C256" s="4">
         <v>81974</v>
@@ -5199,10 +5202,10 @@
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
-        <v>285</v>
+        <v>382</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>287</v>
+        <v>264</v>
       </c>
       <c r="C257" s="4">
         <v>81975</v>
@@ -5213,10 +5216,10 @@
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" s="3" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="B258" s="5" t="s">
-        <v>289</v>
+        <v>266</v>
       </c>
       <c r="C258" s="4">
         <v>81976</v>
@@ -5227,10 +5230,10 @@
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" s="3" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>291</v>
+        <v>268</v>
       </c>
       <c r="C259" s="4">
         <v>81985</v>
@@ -5241,10 +5244,10 @@
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" s="3" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="C260" s="4">
         <v>81986</v>
@@ -5255,10 +5258,10 @@
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" s="3" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>292</v>
+        <v>269</v>
       </c>
       <c r="C261" s="4">
         <v>81978</v>
@@ -5269,10 +5272,10 @@
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" s="3" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="B262" s="5" t="s">
-        <v>293</v>
+        <v>270</v>
       </c>
       <c r="C262" s="4">
         <v>81987</v>
@@ -5283,10 +5286,10 @@
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="B263" s="5" t="s">
-        <v>294</v>
+        <v>271</v>
       </c>
       <c r="C263" s="4">
         <v>81988</v>
@@ -5297,10 +5300,10 @@
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" s="3" t="s">
-        <v>295</v>
+        <v>383</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>296</v>
+        <v>272</v>
       </c>
       <c r="C264" s="4">
         <v>81024</v>
@@ -5311,10 +5314,10 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" s="3" t="s">
-        <v>297</v>
+        <v>384</v>
       </c>
       <c r="B265" s="5" t="s">
-        <v>298</v>
+        <v>273</v>
       </c>
       <c r="C265" s="4">
         <v>81917</v>
@@ -5325,10 +5328,10 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" s="3" t="s">
-        <v>297</v>
+        <v>384</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>299</v>
+        <v>274</v>
       </c>
       <c r="C266" s="4">
         <v>81918</v>
@@ -5339,10 +5342,10 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" s="3" t="s">
-        <v>297</v>
+        <v>384</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>300</v>
+        <v>275</v>
       </c>
       <c r="C267" s="4">
         <v>81919</v>
@@ -5353,10 +5356,10 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" s="3" t="s">
-        <v>297</v>
+        <v>384</v>
       </c>
       <c r="B268" s="5" t="s">
-        <v>301</v>
+        <v>276</v>
       </c>
       <c r="C268" s="4">
         <v>81920</v>

</xml_diff>

<commit_message>
change the color of category
</commit_message>
<xml_diff>
--- a/backyard_list.xlsx
+++ b/backyard_list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyApp\orderapp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\orderapp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EFA228E-1510-46BA-8717-C423BA25D379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BA3B9AE-8792-4783-829C-6B126B330671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4A8513A4-3F40-4E3B-8380-35919E37163E}"/>
+    <workbookView xWindow="18960" yWindow="1210" windowWidth="18510" windowHeight="20250" xr2:uid="{4A8513A4-3F40-4E3B-8380-35919E37163E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -470,9 +470,6 @@
     <t>ELIXIR DISPLAY SET(18)</t>
   </si>
   <si>
-    <t>VIA Free Style</t>
-  </si>
-  <si>
     <t>Braiding Mousse 8oz</t>
   </si>
   <si>
@@ -509,9 +506,6 @@
     <t>30 Eyelash WH 0.25&amp;1oz glu</t>
   </si>
   <si>
-    <t>Beard Guyz</t>
-  </si>
-  <si>
     <t>Beard Wash 8 oz</t>
   </si>
   <si>
@@ -785,9 +779,6 @@
     <t>SM 12 pc Display Set</t>
   </si>
   <si>
-    <t>Groganics</t>
-  </si>
-  <si>
     <t>Gro Hair Gro N Wild 6oz</t>
   </si>
   <si>
@@ -803,9 +794,6 @@
     <t>Gro Shampoo 8.5oz (4pcs)</t>
   </si>
   <si>
-    <t>JML Braids your way</t>
-  </si>
-  <si>
     <t>JML Braid Mousse 8oz</t>
   </si>
   <si>
@@ -833,9 +821,6 @@
     <t>JML Boho 1oz &amp; BYW Mousse</t>
   </si>
   <si>
-    <t>JML Boho Styles &amp; Trends</t>
-  </si>
-  <si>
     <t>JML Boho Detangler 4oz (12)</t>
   </si>
   <si>
@@ -1103,94 +1088,109 @@
     <t>SP HAIR BONDING GLUE</t>
   </si>
   <si>
-    <t>AE Spritz</t>
-  </si>
-  <si>
-    <t>AE Shine/Herbal Oil</t>
-  </si>
-  <si>
-    <t>AE Lotion/Shampoo/Spray</t>
-  </si>
-  <si>
-    <t>SP BRAID SHEEN Shine Spray</t>
-  </si>
-  <si>
     <t>SP HAIR FOOD</t>
   </si>
   <si>
     <t>30 LACE BOND REMOVER</t>
   </si>
   <si>
-    <t>30 Eyelash Glue</t>
-  </si>
-  <si>
-    <t>30 Eyelash Glue 0.25oz Tube</t>
-  </si>
-  <si>
-    <t>VIA Oil-Free WIG SHINE</t>
-  </si>
-  <si>
-    <t>VIA Tube Oil 24pc</t>
-  </si>
-  <si>
-    <t>VIA Tube Oil 3.5oz</t>
-  </si>
-  <si>
     <t>VIA BRAIDING SHINE JELO</t>
   </si>
   <si>
-    <t>VIA Premium Elixir Oil</t>
-  </si>
-  <si>
     <t>VIA PREMIUM STYLING GELS</t>
   </si>
   <si>
-    <t>JML Wax and Gel</t>
-  </si>
-  <si>
-    <t>JML Loc Unloc</t>
-  </si>
-  <si>
-    <t>JML Cactus</t>
-  </si>
-  <si>
-    <t>JML Sp/Lo/Sh/Con</t>
-  </si>
-  <si>
-    <t>SP REMOVER LO/SH</t>
-  </si>
-  <si>
-    <t>30 Sec Eyelash &amp; Glue Combo</t>
-  </si>
-  <si>
-    <t>JML JBCO Sh/Con</t>
-  </si>
-  <si>
-    <t>NEW JML BCO 2oz</t>
-  </si>
-  <si>
     <t>JML BCO 4oz</t>
   </si>
   <si>
     <t>JML BCO 8oz</t>
   </si>
   <si>
-    <t>JML Minis Travel Size</t>
-  </si>
-  <si>
-    <t>Robert Diamond</t>
-  </si>
-  <si>
-    <t>Smooth Moisture</t>
-  </si>
-  <si>
-    <t>JML Boho &amp; BYW Combo</t>
-  </si>
-  <si>
-    <t>JML Island Oil Gels 20oz</t>
-  </si>
-  <si>
-    <t>Hot Water Braid Dipper Jar</t>
+    <t>30 EYELASH GLUE 0.25oz TUBE</t>
+  </si>
+  <si>
+    <t>AE SPRITZ</t>
+  </si>
+  <si>
+    <t>AE SHINE / HERBAL OIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP BRAID SHEEN SHINE SPRAY </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIA OIL-FREE WIG SHINE </t>
+  </si>
+  <si>
+    <t>VIA TUBE OIL 24pc</t>
+  </si>
+  <si>
+    <t>VIA TUBE OIL 3.5oz</t>
+  </si>
+  <si>
+    <t>VIA PREMIUM ELIXIR OIL</t>
+  </si>
+  <si>
+    <t>VIA FREE STYLE</t>
+  </si>
+  <si>
+    <t>BEARD GUYZ</t>
+  </si>
+  <si>
+    <t>JML WAX AND GEL</t>
+  </si>
+  <si>
+    <t>JML LOC UNLOC</t>
+  </si>
+  <si>
+    <t>JML CACTUS</t>
+  </si>
+  <si>
+    <t>30 EYELASH 0.25 &amp; 1oz GLUE COMBO</t>
+  </si>
+  <si>
+    <t>JML MINIS TRAVEL SIZE</t>
+  </si>
+  <si>
+    <t>ROBERT DIAMOND</t>
+  </si>
+  <si>
+    <t>SMOOTH MOISTURE</t>
+  </si>
+  <si>
+    <t>GROGANICS</t>
+  </si>
+  <si>
+    <t>JML BRAIDS YOUR WAY</t>
+  </si>
+  <si>
+    <t>JML BOHO &amp; BYW COMBO</t>
+  </si>
+  <si>
+    <t>JML BOHO STYLES &amp; TRENDS</t>
+  </si>
+  <si>
+    <t>JML ISLAND OIL GELS 20oz</t>
+  </si>
+  <si>
+    <t>Hot WATER BRAID DIPPER JAR</t>
+  </si>
+  <si>
+    <t>JML SPR / LOT / SHAMP / COND</t>
+  </si>
+  <si>
+    <t>JML JBCO SHAMP / COND</t>
+  </si>
+  <si>
+    <t>JML BCO 2oz</t>
+  </si>
+  <si>
+    <t>AE LOT / SHAMP / SPR</t>
+  </si>
+  <si>
+    <t>SP REMOVER LOT / SHAMP</t>
+  </si>
+  <si>
+    <t>30 EYELASH GLUE 1dz</t>
   </si>
 </sst>
 </file>
@@ -1608,31 +1608,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FAE592D-BB12-4B90-B5C8-3064949F562A}">
   <dimension ref="A1:D268"/>
-  <sheetFormatPr defaultColWidth="39" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="39" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>0</v>
@@ -1644,9 +1644,9 @@
         <v>23.04</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>1</v>
@@ -1658,9 +1658,9 @@
         <v>23.04</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -1672,9 +1672,9 @@
         <v>42.24</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>3</v>
@@ -1686,9 +1686,9 @@
         <v>26.27</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>4</v>
@@ -1700,9 +1700,9 @@
         <v>15.18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>5</v>
@@ -1714,9 +1714,9 @@
         <v>18.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
@@ -1728,9 +1728,9 @@
         <v>42.24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>7</v>
@@ -1742,9 +1742,9 @@
         <v>38.4</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>8</v>
@@ -1756,9 +1756,9 @@
         <v>26.88</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>9</v>
@@ -1770,9 +1770,9 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>10</v>
@@ -1784,9 +1784,9 @@
         <v>26.88</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>357</v>
+        <v>382</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>11</v>
@@ -1798,9 +1798,9 @@
         <v>47.75</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>12</v>
@@ -1812,9 +1812,9 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>13</v>
@@ -1826,9 +1826,9 @@
         <v>40.799999999999997</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>14</v>
@@ -1840,9 +1840,9 @@
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>15</v>
@@ -1854,9 +1854,9 @@
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>16</v>
@@ -1868,23 +1868,23 @@
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="D19" s="3">
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>18</v>
@@ -1896,9 +1896,9 @@
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>19</v>
@@ -1910,9 +1910,9 @@
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>20</v>
@@ -1924,9 +1924,9 @@
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>21</v>
@@ -1938,9 +1938,9 @@
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>22</v>
@@ -1952,9 +1952,9 @@
         <v>84.96</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>23</v>
@@ -1966,9 +1966,9 @@
         <v>57.96</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>24</v>
@@ -1980,9 +1980,9 @@
         <v>55.94</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>25</v>
@@ -1994,9 +1994,9 @@
         <v>16.38</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>30</v>
@@ -2008,9 +2008,9 @@
         <v>21.6</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>26</v>
@@ -2022,9 +2022,9 @@
         <v>18.22</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>27</v>
@@ -2036,9 +2036,9 @@
         <v>16.63</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>28</v>
@@ -2050,9 +2050,9 @@
         <v>22.56</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>48</v>
@@ -2064,9 +2064,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -2078,9 +2078,9 @@
         <v>31.75</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>32</v>
@@ -2092,9 +2092,9 @@
         <v>61.44</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>33</v>
@@ -2106,9 +2106,9 @@
         <v>40.32</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>34</v>
@@ -2120,9 +2120,9 @@
         <v>39.56</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>35</v>
@@ -2134,9 +2134,9 @@
         <v>90.14</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>36</v>
@@ -2148,9 +2148,9 @@
         <v>58.24</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>37</v>
@@ -2162,9 +2162,9 @@
         <v>53.92</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>38</v>
@@ -2176,9 +2176,9 @@
         <v>80.260000000000005</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>39</v>
@@ -2190,9 +2190,9 @@
         <v>57.76</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>11</v>
@@ -2204,9 +2204,9 @@
         <v>40.72</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>40</v>
@@ -2218,9 +2218,9 @@
         <v>22.47</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>41</v>
@@ -2232,9 +2232,9 @@
         <v>76.8</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>42</v>
@@ -2246,9 +2246,9 @@
         <v>57.76</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>43</v>
@@ -2260,9 +2260,9 @@
         <v>35.36</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>44</v>
@@ -2274,9 +2274,9 @@
         <v>45.36</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>45</v>
@@ -2288,9 +2288,9 @@
         <v>34.78</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>46</v>
@@ -2302,9 +2302,9 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>47</v>
@@ -2316,9 +2316,9 @@
         <v>119.09</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>49</v>
@@ -2330,9 +2330,9 @@
         <v>26.96</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>50</v>
@@ -2344,9 +2344,9 @@
         <v>29.12</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>51</v>
@@ -2358,7 +2358,7 @@
         <v>53.92</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>52</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>46.08</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
         <v>52</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>41.94</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>52</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>46.08</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
         <v>52</v>
       </c>
@@ -2414,9 +2414,9 @@
         <v>41.94</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>361</v>
+        <v>384</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>57</v>
@@ -2428,9 +2428,9 @@
         <v>118.8</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>361</v>
+        <v>384</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>58</v>
@@ -2442,9 +2442,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>361</v>
+        <v>384</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>59</v>
@@ -2456,9 +2456,9 @@
         <v>118.8</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>361</v>
+        <v>384</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>60</v>
@@ -2470,9 +2470,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>61</v>
@@ -2484,9 +2484,9 @@
         <v>42.84</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>62</v>
@@ -2498,7 +2498,7 @@
         <v>42.84</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
         <v>63</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>77.040000000000006</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
         <v>63</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>38.479999999999997</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
         <v>63</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>77.040000000000006</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
         <v>63</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>67.36</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
         <v>68</v>
       </c>
@@ -2562,13 +2562,13 @@
         <v>69</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="D68" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
         <v>68</v>
       </c>
@@ -2576,13 +2576,13 @@
         <v>70</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="D69" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
         <v>68</v>
       </c>
@@ -2590,13 +2590,13 @@
         <v>71</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="D70" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
         <v>68</v>
       </c>
@@ -2604,13 +2604,13 @@
         <v>72</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="D71" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>68</v>
       </c>
@@ -2618,13 +2618,13 @@
         <v>73</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="D72" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
         <v>68</v>
       </c>
@@ -2632,13 +2632,13 @@
         <v>74</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="D73" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
         <v>68</v>
       </c>
@@ -2646,13 +2646,13 @@
         <v>75</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="D74" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>68</v>
       </c>
@@ -2660,13 +2660,13 @@
         <v>76</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D75" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
         <v>68</v>
       </c>
@@ -2674,13 +2674,13 @@
         <v>77</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="D76" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
         <v>68</v>
       </c>
@@ -2688,13 +2688,13 @@
         <v>78</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="D77" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
         <v>68</v>
       </c>
@@ -2702,13 +2702,13 @@
         <v>79</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="D78" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>68</v>
       </c>
@@ -2716,13 +2716,13 @@
         <v>80</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="D79" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>68</v>
       </c>
@@ -2730,13 +2730,13 @@
         <v>81</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="D80" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
         <v>68</v>
       </c>
@@ -2744,13 +2744,13 @@
         <v>82</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="D81" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="3" t="s">
         <v>68</v>
       </c>
@@ -2758,13 +2758,13 @@
         <v>83</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="D82" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
         <v>68</v>
       </c>
@@ -2772,13 +2772,13 @@
         <v>84</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D83" s="3">
         <v>8.34</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
         <v>86</v>
       </c>
@@ -2786,13 +2786,13 @@
         <v>85</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="D84" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
         <v>86</v>
       </c>
@@ -2800,13 +2800,13 @@
         <v>87</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="D85" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
         <v>86</v>
       </c>
@@ -2814,13 +2814,13 @@
         <v>88</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="D86" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
         <v>86</v>
       </c>
@@ -2828,13 +2828,13 @@
         <v>89</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="D87" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
         <v>86</v>
       </c>
@@ -2842,13 +2842,13 @@
         <v>90</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="D88" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
         <v>86</v>
       </c>
@@ -2856,13 +2856,13 @@
         <v>91</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="D89" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="3" t="s">
         <v>86</v>
       </c>
@@ -2870,13 +2870,13 @@
         <v>92</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="D90" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="3" t="s">
         <v>86</v>
       </c>
@@ -2884,13 +2884,13 @@
         <v>93</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="D91" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="3" t="s">
         <v>86</v>
       </c>
@@ -2898,13 +2898,13 @@
         <v>94</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="D92" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="3" t="s">
         <v>86</v>
       </c>
@@ -2912,13 +2912,13 @@
         <v>95</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="D93" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="3" t="s">
         <v>86</v>
       </c>
@@ -2926,13 +2926,13 @@
         <v>96</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D94" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="3" t="s">
         <v>86</v>
       </c>
@@ -2940,13 +2940,13 @@
         <v>97</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="D95" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="3" t="s">
         <v>86</v>
       </c>
@@ -2954,13 +2954,13 @@
         <v>98</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="D96" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="3" t="s">
         <v>86</v>
       </c>
@@ -2968,13 +2968,13 @@
         <v>99</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="D97" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" s="3" t="s">
         <v>86</v>
       </c>
@@ -2982,13 +2982,13 @@
         <v>100</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="D98" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
         <v>86</v>
       </c>
@@ -2996,15 +2996,15 @@
         <v>101</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="D99" s="3">
         <v>14.46</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" s="3" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>102</v>
@@ -3016,9 +3016,9 @@
         <v>51.75</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="3" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>103</v>
@@ -3030,9 +3030,9 @@
         <v>32.43</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="3" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>104</v>
@@ -3044,9 +3044,9 @@
         <v>32.840000000000003</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>105</v>
@@ -3058,9 +3058,9 @@
         <v>51.09</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>106</v>
@@ -3072,9 +3072,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>107</v>
@@ -3086,9 +3086,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>108</v>
@@ -3100,9 +3100,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>130</v>
@@ -3114,9 +3114,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>109</v>
@@ -3128,9 +3128,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>110</v>
@@ -3142,9 +3142,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>111</v>
@@ -3156,9 +3156,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>112</v>
@@ -3170,9 +3170,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>113</v>
@@ -3184,9 +3184,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>114</v>
@@ -3198,9 +3198,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>115</v>
@@ -3212,9 +3212,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>116</v>
@@ -3226,9 +3226,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>117</v>
@@ -3240,9 +3240,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B117" s="6" t="s">
         <v>118</v>
@@ -3254,9 +3254,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>119</v>
@@ -3268,9 +3268,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B119" s="5" t="s">
         <v>120</v>
@@ -3282,9 +3282,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>121</v>
@@ -3296,9 +3296,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B121" s="5" t="s">
         <v>122</v>
@@ -3310,9 +3310,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B122" s="5" t="s">
         <v>123</v>
@@ -3324,9 +3324,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>124</v>
@@ -3338,9 +3338,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>129</v>
@@ -3352,9 +3352,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>125</v>
@@ -3366,9 +3366,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>128</v>
@@ -3380,9 +3380,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B127" s="5" t="s">
         <v>126</v>
@@ -3394,9 +3394,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B128" s="5" t="s">
         <v>131</v>
@@ -3408,9 +3408,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B129" s="5" t="s">
         <v>127</v>
@@ -3422,9 +3422,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B130" s="5" t="s">
         <v>132</v>
@@ -3436,9 +3436,9 @@
         <v>25.44</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" s="3" t="s">
-        <v>366</v>
+        <v>352</v>
       </c>
       <c r="B131" s="5" t="s">
         <v>133</v>
@@ -3450,9 +3450,9 @@
         <v>25.14</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="3" t="s">
-        <v>366</v>
+        <v>352</v>
       </c>
       <c r="B132" s="5" t="s">
         <v>134</v>
@@ -3464,9 +3464,9 @@
         <v>53.36</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" s="3" t="s">
-        <v>366</v>
+        <v>352</v>
       </c>
       <c r="B133" s="5" t="s">
         <v>135</v>
@@ -3478,9 +3478,9 @@
         <v>25.14</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" s="3" t="s">
-        <v>366</v>
+        <v>352</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>136</v>
@@ -3492,9 +3492,9 @@
         <v>53.36</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" s="3" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>137</v>
@@ -3506,9 +3506,9 @@
         <v>21.54</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" s="3" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B136" s="5" t="s">
         <v>138</v>
@@ -3520,9 +3520,9 @@
         <v>21.54</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" s="3" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B137" s="5" t="s">
         <v>139</v>
@@ -3534,9 +3534,9 @@
         <v>21.54</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" s="3" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B138" s="5" t="s">
         <v>140</v>
@@ -3548,9 +3548,9 @@
         <v>21.54</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" s="3" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B139" s="5" t="s">
         <v>141</v>
@@ -3562,9 +3562,9 @@
         <v>21.54</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" s="3" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B140" s="5" t="s">
         <v>142</v>
@@ -3576,9 +3576,9 @@
         <v>21.54</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" s="3" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B141" s="5" t="s">
         <v>143</v>
@@ -3590,12 +3590,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="B142" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="C142" s="4">
         <v>1899</v>
@@ -3604,12 +3604,12 @@
         <v>28.74</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" s="3" t="s">
-        <v>144</v>
+        <v>364</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C143" s="4">
         <v>1900</v>
@@ -3618,12 +3618,12 @@
         <v>28.74</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" s="3" t="s">
-        <v>144</v>
+        <v>364</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C144" s="4">
         <v>1901</v>
@@ -3632,12 +3632,12 @@
         <v>28.74</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" s="3" t="s">
-        <v>144</v>
+        <v>364</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C145" s="4">
         <v>1902</v>
@@ -3646,12 +3646,12 @@
         <v>28.74</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" s="3" t="s">
-        <v>144</v>
+        <v>364</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C146" s="4">
         <v>1903</v>
@@ -3660,12 +3660,12 @@
         <v>28.74</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" s="3" t="s">
-        <v>144</v>
+        <v>364</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C147" s="4">
         <v>1904</v>
@@ -3674,12 +3674,12 @@
         <v>28.74</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" s="3" t="s">
-        <v>144</v>
+        <v>364</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C148" s="4">
         <v>1905</v>
@@ -3688,12 +3688,12 @@
         <v>110.96</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" s="3" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C149" s="4">
         <v>8380</v>
@@ -3702,12 +3702,12 @@
         <v>7.68</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" s="3" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C150" s="4">
         <v>8385</v>
@@ -3716,12 +3716,12 @@
         <v>12.64</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" s="3" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C151" s="4">
         <v>8384</v>
@@ -3730,12 +3730,12 @@
         <v>7.68</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" s="3" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C152" s="4">
         <v>8389</v>
@@ -3744,12 +3744,12 @@
         <v>12.64</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A153" s="5" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C153" s="4">
         <v>24696</v>
@@ -3758,152 +3758,152 @@
         <v>30.04</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A154" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="D154" s="3">
         <v>37.76</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A155" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="B155" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B155" s="5" t="s">
-        <v>159</v>
-      </c>
       <c r="C155" s="4" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="D155" s="3">
         <v>37.76</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B156" s="6" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D156" s="3">
         <v>194.24</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A157" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B157" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D157" s="3">
         <v>194.24</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A158" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="D158" s="3">
         <v>75.52</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A159" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B159" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="D159" s="3">
         <v>194.24</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A160" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="D160" s="3">
         <v>75.52</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B161" s="6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="D161" s="3">
         <v>75.52</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A162" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D162" s="3">
         <v>75.52</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A163" s="3" t="s">
-        <v>157</v>
+        <v>365</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="D163" s="3">
         <v>151.04</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A164" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C164" s="4">
         <v>29080</v>
@@ -3912,12 +3912,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A165" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C165" s="4">
         <v>29085</v>
@@ -3926,12 +3926,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A166" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C166" s="4">
         <v>29401</v>
@@ -3940,12 +3940,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A167" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C167" s="4">
         <v>29402</v>
@@ -3954,12 +3954,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A168" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C168" s="4">
         <v>29420</v>
@@ -3968,12 +3968,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A169" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B169" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C169" s="4">
         <v>29050</v>
@@ -3982,12 +3982,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A170" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B170" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C170" s="4">
         <v>29055</v>
@@ -3996,12 +3996,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B171" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C171" s="4">
         <v>29020</v>
@@ -4010,12 +4010,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A172" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B172" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C172" s="4">
         <v>29010</v>
@@ -4024,12 +4024,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A173" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B173" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C173" s="4">
         <v>29093</v>
@@ -4038,12 +4038,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A174" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B174" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C174" s="4">
         <v>29302</v>
@@ -4052,12 +4052,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A175" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B175" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C175" s="4">
         <v>29407</v>
@@ -4066,12 +4066,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A176" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B176" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C176" s="4">
         <v>29405</v>
@@ -4080,12 +4080,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A177" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B177" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C177" s="4">
         <v>29409</v>
@@ -4094,12 +4094,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A178" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B178" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C178" s="4">
         <v>29030</v>
@@ -4108,12 +4108,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A179" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B179" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C179" s="4">
         <v>29406</v>
@@ -4122,12 +4122,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A180" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B180" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C180" s="4">
         <v>29304</v>
@@ -4136,12 +4136,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A181" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B181" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C181" s="4">
         <v>29300</v>
@@ -4150,12 +4150,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A182" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C182" s="4">
         <v>29060</v>
@@ -4164,12 +4164,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A183" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B183" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C183" s="4">
         <v>29066</v>
@@ -4178,12 +4178,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A184" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B184" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C184" s="4">
         <v>29070</v>
@@ -4192,12 +4192,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A185" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B185" s="5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C185" s="4">
         <v>29076</v>
@@ -4206,12 +4206,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B186" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C186" s="4">
         <v>29040</v>
@@ -4220,12 +4220,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A187" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B187" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C187" s="4">
         <v>29042</v>
@@ -4234,12 +4234,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A188" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B188" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C188" s="4">
         <v>29041</v>
@@ -4248,12 +4248,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A189" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B189" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C189" s="4">
         <v>29043</v>
@@ -4262,12 +4262,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A190" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B190" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C190" s="4">
         <v>29092</v>
@@ -4276,12 +4276,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A191" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B191" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C191" s="4">
         <v>29094</v>
@@ -4290,12 +4290,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A192" s="3" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B192" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C192" s="4">
         <v>29404</v>
@@ -4304,12 +4304,12 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A193" s="3" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B193" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C193" s="4">
         <v>81921</v>
@@ -4318,12 +4318,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A194" s="3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B194" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C194" s="4">
         <v>29098</v>
@@ -4332,12 +4332,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A195" s="3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C195" s="4">
         <v>29095</v>
@@ -4346,12 +4346,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A196" s="3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B196" s="5" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C196" s="4">
         <v>29096</v>
@@ -4360,12 +4360,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A197" s="3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B197" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C197" s="4">
         <v>29097</v>
@@ -4374,418 +4374,418 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A198" s="3" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="B198" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="D198" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A199" s="3" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="B199" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="D199" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A200" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B200" s="5" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="D200" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A201" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B201" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="D201" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A202" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B202" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="D202" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A203" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B203" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="D203" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A204" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B204" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C204" s="4" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D204" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A205" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B205" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="D205" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A206" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B206" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="D206" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A207" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="D207" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A208" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B208" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C208" s="4" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D208" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A209" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B209" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C209" s="4" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="D209" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A210" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B210" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C210" s="4" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D210" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A211" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="D211" s="3">
         <v>20.16</v>
       </c>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A212" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B212" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C212" s="4" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="D212" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A213" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B213" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C213" s="4" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="D213" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A214" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B214" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C214" s="4" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="D214" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C215" s="4" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="D215" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A216" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C216" s="4" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="D216" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A217" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C217" s="4" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="D217" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A218" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D218" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A219" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="D219" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A220" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B220" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="D220" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A221" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B221" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D221" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A222" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="D222" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A223" s="3" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="D223" s="3">
         <v>34.24</v>
       </c>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" s="3" t="s">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="B224" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="D224" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A225" s="3" t="s">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="B225" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="D225" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A226" s="3" t="s">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="B226" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C226" s="4" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D226" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A227" s="3" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C227" s="4">
         <v>81034</v>
@@ -4794,12 +4794,12 @@
         <v>53.94</v>
       </c>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A228" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C228" s="4">
         <v>81925</v>
@@ -4808,12 +4808,12 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A229" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C229" s="4">
         <v>81927</v>
@@ -4822,12 +4822,12 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A230" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B230" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C230" s="4">
         <v>81929</v>
@@ -4836,12 +4836,12 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A231" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B231" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C231" s="4">
         <v>81033</v>
@@ -4850,12 +4850,12 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A232" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B232" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C232" s="4">
         <v>81926</v>
@@ -4864,12 +4864,12 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A233" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C233" s="4">
         <v>81928</v>
@@ -4878,12 +4878,12 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A234" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B234" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C234" s="4">
         <v>81932</v>
@@ -4892,12 +4892,12 @@
         <v>42.96</v>
       </c>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A235" s="3" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C235" s="4">
         <v>3060</v>
@@ -4906,12 +4906,12 @@
         <v>51.68</v>
       </c>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A236" s="3" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="B236" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C236" s="4">
         <v>3062</v>
@@ -4920,12 +4920,12 @@
         <v>53.6</v>
       </c>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A237" s="3" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="B237" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C237" s="4">
         <v>3059</v>
@@ -4934,12 +4934,12 @@
         <v>51.68</v>
       </c>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A238" s="3" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="B238" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C238" s="4">
         <v>3061</v>
@@ -4948,12 +4948,12 @@
         <v>53.6</v>
       </c>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A239" s="3" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C239" s="4">
         <v>1850</v>
@@ -4962,12 +4962,12 @@
         <v>43.86</v>
       </c>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A240" s="3" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="B240" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C240" s="4">
         <v>1851</v>
@@ -4976,12 +4976,12 @@
         <v>43.86</v>
       </c>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A241" s="3" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C241" s="4">
         <v>1852</v>
@@ -4990,12 +4990,12 @@
         <v>43.86</v>
       </c>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A242" s="3" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C242" s="4">
         <v>1853</v>
@@ -5004,12 +5004,12 @@
         <v>37.14</v>
       </c>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A243" s="3" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="B243" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C243" s="4">
         <v>1856</v>
@@ -5018,12 +5018,12 @@
         <v>71.709999999999994</v>
       </c>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A244" s="3" t="s">
-        <v>249</v>
+        <v>373</v>
       </c>
       <c r="B244" s="5" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C244" s="4">
         <v>76081</v>
@@ -5032,12 +5032,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A245" s="3" t="s">
-        <v>249</v>
+        <v>373</v>
       </c>
       <c r="B245" s="5" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C245" s="4">
         <v>76085</v>
@@ -5046,12 +5046,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A246" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="B246" s="5" t="s">
         <v>249</v>
-      </c>
-      <c r="B246" s="5" t="s">
-        <v>252</v>
       </c>
       <c r="C246" s="4">
         <v>76087</v>
@@ -5060,12 +5060,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A247" s="3" t="s">
-        <v>249</v>
+        <v>373</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C247" s="4">
         <v>76082</v>
@@ -5074,12 +5074,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A248" s="3" t="s">
-        <v>249</v>
+        <v>373</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C248" s="4">
         <v>76086</v>
@@ -5088,12 +5088,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A249" s="3" t="s">
-        <v>255</v>
+        <v>374</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="C249" s="4">
         <v>1015</v>
@@ -5102,12 +5102,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A250" s="3" t="s">
-        <v>255</v>
+        <v>374</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C250" s="4">
         <v>1016</v>
@@ -5116,12 +5116,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A251" s="3" t="s">
-        <v>255</v>
+        <v>374</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C251" s="4">
         <v>1017</v>
@@ -5130,12 +5130,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A252" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="B252" s="5" t="s">
         <v>255</v>
-      </c>
-      <c r="B252" s="5" t="s">
-        <v>259</v>
       </c>
       <c r="C252" s="4">
         <v>1022</v>
@@ -5144,12 +5144,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A253" s="3" t="s">
-        <v>255</v>
+        <v>374</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C253" s="4">
         <v>1018</v>
@@ -5158,12 +5158,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A254" s="3" t="s">
-        <v>255</v>
+        <v>374</v>
       </c>
       <c r="B254" s="5" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="C254" s="4">
         <v>1019</v>
@@ -5172,12 +5172,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A255" s="3" t="s">
-        <v>255</v>
+        <v>374</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C255" s="4">
         <v>1020</v>
@@ -5186,12 +5186,12 @@
         <v>110</v>
       </c>
     </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A256" s="3" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="C256" s="4">
         <v>81974</v>
@@ -5200,12 +5200,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A257" s="3" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="C257" s="4">
         <v>81975</v>
@@ -5214,12 +5214,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A258" s="3" t="s">
-        <v>265</v>
+        <v>376</v>
       </c>
       <c r="B258" s="5" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="C258" s="4">
         <v>81976</v>
@@ -5228,12 +5228,12 @@
         <v>43.08</v>
       </c>
     </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A259" s="3" t="s">
-        <v>265</v>
+        <v>376</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="C259" s="4">
         <v>81985</v>
@@ -5242,12 +5242,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A260" s="3" t="s">
-        <v>265</v>
+        <v>376</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="C260" s="4">
         <v>81986</v>
@@ -5256,12 +5256,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A261" s="3" t="s">
-        <v>265</v>
+        <v>376</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="C261" s="4">
         <v>81978</v>
@@ -5270,12 +5270,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A262" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="B262" s="5" t="s">
         <v>265</v>
-      </c>
-      <c r="B262" s="5" t="s">
-        <v>270</v>
       </c>
       <c r="C262" s="4">
         <v>81987</v>
@@ -5284,12 +5284,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A263" s="3" t="s">
-        <v>265</v>
+        <v>376</v>
       </c>
       <c r="B263" s="5" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="C263" s="4">
         <v>81988</v>
@@ -5298,12 +5298,12 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A264" s="3" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C264" s="4">
         <v>81024</v>
@@ -5312,12 +5312,12 @@
         <v>23.04</v>
       </c>
     </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A265" s="3" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="B265" s="5" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="C265" s="4">
         <v>81917</v>
@@ -5326,12 +5326,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A266" s="3" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C266" s="4">
         <v>81918</v>
@@ -5340,12 +5340,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A267" s="3" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C267" s="4">
         <v>81919</v>
@@ -5354,12 +5354,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A268" s="3" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="B268" s="5" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C268" s="4">
         <v>81920</v>

</xml_diff>